<commit_message>
fix for group pr
</commit_message>
<xml_diff>
--- a/backend/templates/pr-template 2p.xlsx
+++ b/backend/templates/pr-template 2p.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\web-opr\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA680B0-BFC8-4403-88A6-1008B5C9E8ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3D5AFC4-4A42-47C1-98B2-948614655CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -403,7 +403,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -508,18 +508,6 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
@@ -532,9 +520,113 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -553,112 +645,17 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1079,26 +1076,26 @@
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="58"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="68"/>
     </row>
     <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="59" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="61"/>
+      <c r="A2" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="70"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="70"/>
+      <c r="E2" s="70"/>
+      <c r="F2" s="71"/>
     </row>
     <row r="3" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="62"/>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="64"/>
+      <c r="A3" s="72"/>
+      <c r="B3" s="73"/>
+      <c r="C3" s="73"/>
+      <c r="D3" s="73"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="74"/>
     </row>
     <row r="4" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
@@ -1106,439 +1103,439 @@
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="27"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="66"/>
+      <c r="D4" s="75"/>
+      <c r="E4" s="75"/>
+      <c r="F4" s="76"/>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="67" t="s">
+      <c r="A5" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="68"/>
+      <c r="B5" s="78"/>
       <c r="C5" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D5" s="5"/>
-      <c r="E5" s="69" t="s">
+      <c r="E5" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="70"/>
+      <c r="F5" s="80"/>
     </row>
     <row r="6" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="51"/>
-      <c r="B6" s="52"/>
+      <c r="A6" s="83"/>
+      <c r="B6" s="84"/>
       <c r="C6" s="6" t="s">
         <v>2</v>
       </c>
       <c r="D6" s="7"/>
-      <c r="E6" s="49" t="s">
+      <c r="E6" s="81" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="50"/>
+      <c r="F6" s="82"/>
     </row>
     <row r="7" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="53" t="s">
+      <c r="A7" s="85" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="55" t="s">
+      <c r="B7" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="55" t="s">
+      <c r="C7" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="55" t="s">
+      <c r="D7" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="55" t="s">
+      <c r="E7" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="55" t="s">
+      <c r="F7" s="52" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="54"/>
-      <c r="B8" s="56"/>
-      <c r="C8" s="56"/>
-      <c r="D8" s="56"/>
-      <c r="E8" s="56"/>
-      <c r="F8" s="56"/>
+      <c r="A8" s="86"/>
+      <c r="B8" s="53"/>
+      <c r="C8" s="53"/>
+      <c r="D8" s="53"/>
+      <c r="E8" s="53"/>
+      <c r="F8" s="53"/>
     </row>
     <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="46"/>
-      <c r="B9" s="47"/>
-      <c r="C9" s="45"/>
-      <c r="D9" s="45"/>
-      <c r="E9" s="48"/>
+      <c r="A9" s="42"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="87"/>
       <c r="F9" s="39">
         <f t="shared" ref="F9:F42" si="0">D9*E9</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="46"/>
-      <c r="B10" s="47"/>
-      <c r="C10" s="45"/>
-      <c r="D10" s="45"/>
-      <c r="E10" s="48"/>
+      <c r="A10" s="42"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="41"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="87"/>
       <c r="F10" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="46"/>
-      <c r="B11" s="47"/>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="48"/>
+      <c r="A11" s="42"/>
+      <c r="B11" s="43"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="87"/>
       <c r="F11" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="46"/>
-      <c r="B12" s="47"/>
-      <c r="C12" s="45"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="48"/>
+      <c r="A12" s="42"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="87"/>
       <c r="F12" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="46"/>
-      <c r="B13" s="47"/>
-      <c r="C13" s="45"/>
-      <c r="D13" s="45"/>
-      <c r="E13" s="48"/>
+      <c r="A13" s="42"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="41"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="87"/>
       <c r="F13" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="46"/>
-      <c r="B14" s="47"/>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="48"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="43"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="41"/>
+      <c r="E14" s="87"/>
       <c r="F14" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="46"/>
-      <c r="B15" s="47"/>
-      <c r="C15" s="45"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="48"/>
+      <c r="A15" s="42"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="87"/>
       <c r="F15" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="46"/>
-      <c r="B16" s="47"/>
-      <c r="C16" s="45"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="48"/>
+      <c r="A16" s="42"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="87"/>
       <c r="F16" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="46"/>
-      <c r="B17" s="47"/>
-      <c r="C17" s="45"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="48"/>
+      <c r="A17" s="42"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="87"/>
       <c r="F17" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="46"/>
-      <c r="B18" s="47"/>
-      <c r="C18" s="45"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="48"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="87"/>
       <c r="F18" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="46"/>
-      <c r="B19" s="47"/>
-      <c r="C19" s="45"/>
-      <c r="D19" s="45"/>
-      <c r="E19" s="48"/>
+      <c r="A19" s="42"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="41"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="87"/>
       <c r="F19" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="46"/>
-      <c r="B20" s="47"/>
-      <c r="C20" s="45"/>
-      <c r="D20" s="45"/>
-      <c r="E20" s="48"/>
+      <c r="A20" s="42"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="41"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="87"/>
       <c r="F20" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="46"/>
-      <c r="B21" s="47"/>
-      <c r="C21" s="45"/>
-      <c r="D21" s="45"/>
-      <c r="E21" s="48"/>
+      <c r="A21" s="42"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="87"/>
       <c r="F21" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="46"/>
-      <c r="B22" s="47"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="48"/>
+      <c r="A22" s="42"/>
+      <c r="B22" s="43"/>
+      <c r="C22" s="41"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="87"/>
       <c r="F22" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="46"/>
-      <c r="B23" s="47"/>
-      <c r="C23" s="45"/>
-      <c r="D23" s="45"/>
-      <c r="E23" s="48"/>
+      <c r="A23" s="42"/>
+      <c r="B23" s="43"/>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="87"/>
       <c r="F23" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="46"/>
-      <c r="B24" s="47"/>
-      <c r="C24" s="45"/>
-      <c r="D24" s="45"/>
-      <c r="E24" s="48"/>
+      <c r="A24" s="42"/>
+      <c r="B24" s="43"/>
+      <c r="C24" s="41"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="87"/>
       <c r="F24" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="46"/>
-      <c r="B25" s="47"/>
-      <c r="C25" s="45"/>
-      <c r="D25" s="45"/>
-      <c r="E25" s="48"/>
+      <c r="A25" s="42"/>
+      <c r="B25" s="43"/>
+      <c r="C25" s="41"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="87"/>
       <c r="F25" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="46"/>
-      <c r="B26" s="47"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="48"/>
+      <c r="A26" s="42"/>
+      <c r="B26" s="43"/>
+      <c r="C26" s="41"/>
+      <c r="D26" s="41"/>
+      <c r="E26" s="87"/>
       <c r="F26" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="46"/>
-      <c r="B27" s="47"/>
-      <c r="C27" s="45"/>
-      <c r="D27" s="45"/>
-      <c r="E27" s="48"/>
+      <c r="A27" s="42"/>
+      <c r="B27" s="43"/>
+      <c r="C27" s="41"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="87"/>
       <c r="F27" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="46"/>
-      <c r="B28" s="47"/>
-      <c r="C28" s="45"/>
-      <c r="D28" s="45"/>
-      <c r="E28" s="48"/>
+      <c r="A28" s="42"/>
+      <c r="B28" s="43"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="87"/>
       <c r="F28" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="46"/>
-      <c r="B29" s="47"/>
-      <c r="C29" s="45"/>
-      <c r="D29" s="45"/>
-      <c r="E29" s="48"/>
+      <c r="A29" s="42"/>
+      <c r="B29" s="43"/>
+      <c r="C29" s="41"/>
+      <c r="D29" s="41"/>
+      <c r="E29" s="87"/>
       <c r="F29" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="46"/>
-      <c r="B30" s="47"/>
-      <c r="C30" s="45"/>
-      <c r="D30" s="45"/>
-      <c r="E30" s="48"/>
+      <c r="A30" s="42"/>
+      <c r="B30" s="43"/>
+      <c r="C30" s="41"/>
+      <c r="D30" s="41"/>
+      <c r="E30" s="87"/>
       <c r="F30" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="46"/>
-      <c r="B31" s="47"/>
-      <c r="C31" s="45"/>
-      <c r="D31" s="45"/>
-      <c r="E31" s="48"/>
+      <c r="A31" s="42"/>
+      <c r="B31" s="43"/>
+      <c r="C31" s="41"/>
+      <c r="D31" s="41"/>
+      <c r="E31" s="87"/>
       <c r="F31" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="46"/>
-      <c r="B32" s="47"/>
-      <c r="C32" s="45"/>
-      <c r="D32" s="45"/>
-      <c r="E32" s="48"/>
+      <c r="A32" s="42"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="41"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="87"/>
       <c r="F32" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="46"/>
-      <c r="B33" s="47"/>
-      <c r="C33" s="45"/>
-      <c r="D33" s="45"/>
-      <c r="E33" s="48"/>
+      <c r="A33" s="42"/>
+      <c r="B33" s="43"/>
+      <c r="C33" s="41"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="87"/>
       <c r="F33" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="46"/>
-      <c r="B34" s="47"/>
-      <c r="C34" s="45"/>
-      <c r="D34" s="45"/>
-      <c r="E34" s="48"/>
+      <c r="A34" s="42"/>
+      <c r="B34" s="43"/>
+      <c r="C34" s="41"/>
+      <c r="D34" s="41"/>
+      <c r="E34" s="87"/>
       <c r="F34" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="46"/>
-      <c r="B35" s="47"/>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="48"/>
+      <c r="A35" s="42"/>
+      <c r="B35" s="43"/>
+      <c r="C35" s="41"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="87"/>
       <c r="F35" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="46"/>
-      <c r="B36" s="47"/>
-      <c r="C36" s="45"/>
-      <c r="D36" s="45"/>
-      <c r="E36" s="48"/>
+      <c r="A36" s="42"/>
+      <c r="B36" s="43"/>
+      <c r="C36" s="41"/>
+      <c r="D36" s="41"/>
+      <c r="E36" s="87"/>
       <c r="F36" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="46"/>
-      <c r="B37" s="47"/>
-      <c r="C37" s="45"/>
-      <c r="D37" s="45"/>
-      <c r="E37" s="48"/>
+      <c r="A37" s="42"/>
+      <c r="B37" s="43"/>
+      <c r="C37" s="41"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="87"/>
       <c r="F37" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="46"/>
-      <c r="B38" s="47"/>
-      <c r="C38" s="45"/>
-      <c r="D38" s="45"/>
-      <c r="E38" s="48"/>
+      <c r="A38" s="42"/>
+      <c r="B38" s="43"/>
+      <c r="C38" s="41"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="87"/>
       <c r="F38" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G38" s="91" t="s">
+      <c r="G38" s="44" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="46"/>
-      <c r="B39" s="47"/>
-      <c r="C39" s="45"/>
-      <c r="D39" s="45"/>
-      <c r="E39" s="48"/>
+      <c r="A39" s="42"/>
+      <c r="B39" s="43"/>
+      <c r="C39" s="41"/>
+      <c r="D39" s="41"/>
+      <c r="E39" s="87"/>
       <c r="F39" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G39" s="91" t="s">
+      <c r="G39" s="44" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="46"/>
-      <c r="B40" s="47"/>
-      <c r="C40" s="45"/>
-      <c r="D40" s="45"/>
-      <c r="E40" s="48"/>
+      <c r="A40" s="42"/>
+      <c r="B40" s="43"/>
+      <c r="C40" s="41"/>
+      <c r="D40" s="41"/>
+      <c r="E40" s="87"/>
       <c r="F40" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="46"/>
-      <c r="B41" s="47"/>
-      <c r="C41" s="45"/>
-      <c r="D41" s="45"/>
-      <c r="E41" s="48"/>
+      <c r="A41" s="42"/>
+      <c r="B41" s="43"/>
+      <c r="C41" s="41"/>
+      <c r="D41" s="41"/>
+      <c r="E41" s="87"/>
       <c r="F41" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="46"/>
-      <c r="B42" s="47"/>
-      <c r="C42" s="45"/>
-      <c r="D42" s="45"/>
-      <c r="E42" s="48"/>
+      <c r="A42" s="42"/>
+      <c r="B42" s="43"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="41"/>
+      <c r="E42" s="87"/>
       <c r="F42" s="39">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1549,7 +1546,7 @@
       <c r="B43" s="28"/>
       <c r="C43" s="34"/>
       <c r="D43" s="29"/>
-      <c r="E43" s="42"/>
+      <c r="E43" s="88"/>
       <c r="F43" s="39">
         <f t="shared" ref="F43:F68" si="1">D43*E43</f>
         <v>0</v>
@@ -1560,7 +1557,7 @@
       <c r="B44" s="23"/>
       <c r="C44" s="10"/>
       <c r="D44" s="23"/>
-      <c r="E44" s="43"/>
+      <c r="E44" s="89"/>
       <c r="F44" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1571,7 +1568,7 @@
       <c r="B45" s="23"/>
       <c r="C45" s="10"/>
       <c r="D45" s="30"/>
-      <c r="E45" s="43"/>
+      <c r="E45" s="89"/>
       <c r="F45" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1582,7 +1579,7 @@
       <c r="B46" s="23"/>
       <c r="C46" s="10"/>
       <c r="D46" s="30"/>
-      <c r="E46" s="43"/>
+      <c r="E46" s="89"/>
       <c r="F46" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1593,7 +1590,7 @@
       <c r="B47" s="23"/>
       <c r="C47" s="10"/>
       <c r="D47" s="30"/>
-      <c r="E47" s="43"/>
+      <c r="E47" s="89"/>
       <c r="F47" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1604,7 +1601,7 @@
       <c r="B48" s="23"/>
       <c r="C48" s="10"/>
       <c r="D48" s="30"/>
-      <c r="E48" s="43"/>
+      <c r="E48" s="89"/>
       <c r="F48" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1615,7 +1612,7 @@
       <c r="B49" s="23"/>
       <c r="C49" s="35"/>
       <c r="D49" s="30"/>
-      <c r="E49" s="43"/>
+      <c r="E49" s="89"/>
       <c r="F49" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1626,7 +1623,7 @@
       <c r="B50" s="23"/>
       <c r="C50" s="10"/>
       <c r="D50" s="30"/>
-      <c r="E50" s="43"/>
+      <c r="E50" s="89"/>
       <c r="F50" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1637,7 +1634,7 @@
       <c r="B51" s="23"/>
       <c r="C51" s="10"/>
       <c r="D51" s="30"/>
-      <c r="E51" s="43"/>
+      <c r="E51" s="89"/>
       <c r="F51" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1648,7 +1645,7 @@
       <c r="B52" s="23"/>
       <c r="C52" s="10"/>
       <c r="D52" s="30"/>
-      <c r="E52" s="43"/>
+      <c r="E52" s="89"/>
       <c r="F52" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1659,7 +1656,7 @@
       <c r="B53" s="23"/>
       <c r="C53" s="10"/>
       <c r="D53" s="30"/>
-      <c r="E53" s="40"/>
+      <c r="E53" s="90"/>
       <c r="F53" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1670,7 +1667,7 @@
       <c r="B54" s="32"/>
       <c r="C54" s="31"/>
       <c r="D54" s="32"/>
-      <c r="E54" s="44"/>
+      <c r="E54" s="40"/>
       <c r="F54" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1681,7 +1678,7 @@
       <c r="B55" s="32"/>
       <c r="C55" s="31"/>
       <c r="D55" s="32"/>
-      <c r="E55" s="44"/>
+      <c r="E55" s="40"/>
       <c r="F55" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1692,7 +1689,7 @@
       <c r="B56" s="33"/>
       <c r="C56" s="36"/>
       <c r="D56" s="30"/>
-      <c r="E56" s="41"/>
+      <c r="E56" s="87"/>
       <c r="F56" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1703,7 +1700,7 @@
       <c r="B57" s="25"/>
       <c r="C57" s="10"/>
       <c r="D57" s="30"/>
-      <c r="E57" s="40"/>
+      <c r="E57" s="90"/>
       <c r="F57" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1714,7 +1711,7 @@
       <c r="B58" s="25"/>
       <c r="C58" s="10"/>
       <c r="D58" s="30"/>
-      <c r="E58" s="40"/>
+      <c r="E58" s="90"/>
       <c r="F58" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1725,7 +1722,7 @@
       <c r="B59" s="25"/>
       <c r="C59" s="37"/>
       <c r="D59" s="30"/>
-      <c r="E59" s="40"/>
+      <c r="E59" s="90"/>
       <c r="F59" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1736,7 +1733,7 @@
       <c r="B60" s="25"/>
       <c r="C60" s="10"/>
       <c r="D60" s="30"/>
-      <c r="E60" s="40"/>
+      <c r="E60" s="90"/>
       <c r="F60" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1747,7 +1744,7 @@
       <c r="B61" s="24"/>
       <c r="C61" s="10"/>
       <c r="D61" s="30"/>
-      <c r="E61" s="40"/>
+      <c r="E61" s="90"/>
       <c r="F61" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1758,7 +1755,7 @@
       <c r="B62" s="24"/>
       <c r="C62" s="10"/>
       <c r="D62" s="30"/>
-      <c r="E62" s="40"/>
+      <c r="E62" s="90"/>
       <c r="F62" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1769,7 +1766,7 @@
       <c r="B63" s="24"/>
       <c r="C63" s="10"/>
       <c r="D63" s="30"/>
-      <c r="E63" s="40"/>
+      <c r="E63" s="90"/>
       <c r="F63" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1780,7 +1777,7 @@
       <c r="B64" s="24"/>
       <c r="C64" s="10"/>
       <c r="D64" s="30"/>
-      <c r="E64" s="40"/>
+      <c r="E64" s="90"/>
       <c r="F64" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1791,7 +1788,7 @@
       <c r="B65" s="24"/>
       <c r="C65" s="10"/>
       <c r="D65" s="30"/>
-      <c r="E65" s="40"/>
+      <c r="E65" s="90"/>
       <c r="F65" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1802,7 +1799,7 @@
       <c r="B66" s="11"/>
       <c r="C66" s="37"/>
       <c r="D66" s="30"/>
-      <c r="E66" s="40"/>
+      <c r="E66" s="90"/>
       <c r="F66" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1813,7 +1810,7 @@
       <c r="B67" s="11"/>
       <c r="C67" s="37"/>
       <c r="D67" s="30"/>
-      <c r="E67" s="40"/>
+      <c r="E67" s="90"/>
       <c r="F67" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1824,7 +1821,7 @@
       <c r="B68" s="11"/>
       <c r="C68" s="37"/>
       <c r="D68" s="38"/>
-      <c r="E68" s="40"/>
+      <c r="E68" s="90"/>
       <c r="F68" s="39">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1834,44 +1831,44 @@
       <c r="A69" s="12"/>
       <c r="B69" s="13"/>
       <c r="C69" s="14"/>
-      <c r="D69" s="78" t="s">
+      <c r="D69" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="E69" s="79"/>
+      <c r="E69" s="55"/>
       <c r="F69" s="9">
         <f>SUM(F9:F68)</f>
         <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="88" t="s">
+      <c r="A70" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="B70" s="89"/>
-      <c r="C70" s="89"/>
-      <c r="D70" s="89"/>
-      <c r="E70" s="89"/>
-      <c r="F70" s="90"/>
+      <c r="B70" s="65"/>
+      <c r="C70" s="65"/>
+      <c r="D70" s="65"/>
+      <c r="E70" s="65"/>
+      <c r="F70" s="66"/>
     </row>
     <row r="71" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A71" s="80"/>
-      <c r="B71" s="81"/>
-      <c r="C71" s="81"/>
-      <c r="D71" s="81"/>
-      <c r="E71" s="81"/>
-      <c r="F71" s="82"/>
+      <c r="A71" s="56"/>
+      <c r="B71" s="57"/>
+      <c r="C71" s="57"/>
+      <c r="D71" s="57"/>
+      <c r="E71" s="57"/>
+      <c r="F71" s="58"/>
     </row>
     <row r="72" spans="1:7" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="83" t="s">
+      <c r="A72" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="B72" s="84"/>
-      <c r="C72" s="85"/>
-      <c r="D72" s="86" t="s">
+      <c r="B72" s="60"/>
+      <c r="C72" s="61"/>
+      <c r="D72" s="62" t="s">
         <v>11</v>
       </c>
-      <c r="E72" s="86"/>
-      <c r="F72" s="87"/>
+      <c r="E72" s="62"/>
+      <c r="F72" s="63"/>
     </row>
     <row r="73" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="3" t="s">
@@ -1879,9 +1876,9 @@
       </c>
       <c r="B73" s="15"/>
       <c r="C73" s="21"/>
-      <c r="D73" s="71"/>
-      <c r="E73" s="72"/>
-      <c r="F73" s="73"/>
+      <c r="D73" s="45"/>
+      <c r="E73" s="46"/>
+      <c r="F73" s="47"/>
     </row>
     <row r="74" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
@@ -1889,9 +1886,9 @@
       </c>
       <c r="B74" s="15"/>
       <c r="C74" s="16"/>
-      <c r="D74" s="74"/>
-      <c r="E74" s="74"/>
-      <c r="F74" s="75"/>
+      <c r="D74" s="48"/>
+      <c r="E74" s="48"/>
+      <c r="F74" s="49"/>
     </row>
     <row r="75" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="17" t="s">
@@ -1899,12 +1896,12 @@
       </c>
       <c r="B75" s="18"/>
       <c r="C75" s="22"/>
-      <c r="D75" s="76" t="s">
+      <c r="D75" s="50" t="s">
         <v>15</v>
       </c>
-      <c r="E75" s="76"/>
-      <c r="F75" s="77"/>
-      <c r="G75" s="91" t="s">
+      <c r="E75" s="50"/>
+      <c r="F75" s="51"/>
+      <c r="G75" s="44" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1915,7 +1912,7 @@
       <c r="D76" s="19"/>
       <c r="E76" s="19"/>
       <c r="F76" s="20"/>
-      <c r="G76" s="91" t="s">
+      <c r="G76" s="44" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1924,6 +1921,18 @@
     <sortCondition ref="K6:K56"/>
   </sortState>
   <mergeCells count="23">
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="E5:F5"/>
     <mergeCell ref="D73:F73"/>
     <mergeCell ref="D74:F74"/>
     <mergeCell ref="D75:F75"/>
@@ -1935,18 +1944,6 @@
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="A70:B70"/>
     <mergeCell ref="C70:F70"/>
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="1.7716535433070868" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="91" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>